<commit_message>
Update index: 9941 → 9969 [scan complete]
Scanned 29 addresses from index 9941 to 9969.
Found 1 confirmed business: אטיאס אברהם (רו"ח) at הרב הרצוג 83, ירושלים.
Updated Excel report for 29-07-2026.
</commit_message>
<xml_diff>
--- a/excel outputs/דוח נכסים לתאריך:29-07-2026.xlsx
+++ b/excel outputs/דוח נכסים לתאריך:29-07-2026.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="נכסים חשודים" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ממצאים" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,9 +29,20 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -41,11 +52,15 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
-        <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -53,14 +68,34 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="001F4E79"/>
+      </left>
+      <right style="thin">
+        <color rgb="001F4E79"/>
+      </right>
+      <top style="thin">
+        <color rgb="001F4E79"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="001F4E79"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -427,19 +462,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="33" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="41" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>שם העסק</t>
@@ -476,123 +511,44 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>פרנג'י הנדסת חשמל</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>הרב דוד אלטשולר 103, ירושלים</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>חשמלאי / הנדסת חשמל</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>אטיאס אברהם</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>הרב הרצוג 83, ירושלים</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>רואי חשבון ✅</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>גבוה</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80034876/17910/</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>דיג'יי אלוני מיקס</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>הרב דוד אלטשולר 105, ירושלים</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>תקליטן / מוזיקה לאירועים</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80008819/24390/</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>אלוני בלוני</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>הרב דוד אלטשולר 105, ירושלים</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>הפעלות לימי הולדת</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80263931/9010120/</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>מח"פ מכון לפוליגרף - עזר שאול</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>הרב אליעזרי 5, ירושלים</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>מכון פוליגרף / בדיקות כשירות</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/20940840/17200/</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/195210/46140/</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>https://easy.co.il/en/page/25991860</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update index: 9969 → 9979 | scan session 29-07-2026 [round 2]
Scanned addresses 9969-9978 (הרב ז'ולטי בצלאל 10-20)
Found 1 business: קרן פנינה - בגדי גברים (הרב בצלאל זולטי 19)

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016g5yo3d2qEPUpYg65gNYf4
</commit_message>
<xml_diff>
--- a/excel outputs/דוח נכסים לתאריך:29-07-2026.xlsx
+++ b/excel outputs/דוח נכסים לתאריך:29-07-2026.xlsx
@@ -29,16 +29,16 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <color rgb="000563C1"/>
-      <sz val="10"/>
+      <sz val="11"/>
       <u val="single"/>
     </font>
   </fonts>
@@ -52,11 +52,13 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -70,16 +72,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="001F4E79"/>
+        <color rgb="00CCCCCC"/>
       </left>
       <right style="thin">
-        <color rgb="001F4E79"/>
+        <color rgb="00CCCCCC"/>
       </right>
       <top style="thin">
-        <color rgb="001F4E79"/>
+        <color rgb="00CCCCCC"/>
       </top>
       <bottom style="thin">
-        <color rgb="001F4E79"/>
+        <color rgb="00CCCCCC"/>
       </bottom>
     </border>
   </borders>
@@ -94,7 +96,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -468,13 +470,13 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="35" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>שם העסק</t>
@@ -511,20 +513,20 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1">
+    <row r="2" ht="25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>אטיאס אברהם</t>
+          <t>קרן פנינה - בגדי גברים</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>הרב הרצוג 83, ירושלים</t>
+          <t>הרב בצלאל זולטי 19, ירושלים</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>רואי חשבון ✅</t>
+          <t>בגדי גברים</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -534,21 +536,13 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>https://www.d.co.il/195210/46140/</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>https://easy.co.il/en/page/25991860</t>
-        </is>
-      </c>
+          <t>https://www.b144.co.il/b144_sip/401C04134171675849140116/</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId2"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>